<commit_message>
Hoan thanh In checksheet ra excel
</commit_message>
<xml_diff>
--- a/TWSL/TEMP/TEMP.xlsx
+++ b/TWSL/TEMP/TEMP.xlsx
@@ -5,16 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\249533\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\4.DEV\C#\TWSL\TWSL\TEMP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F0FF6DB-5A38-43B4-A3EA-F384CBEF90EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1183C3-291A-4593-BB04-892DF5500EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4A80FBE-14A8-425E-A0AC-B410392117A6}"/>
+    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{B4A80FBE-14A8-425E-A0AC-B410392117A6}"/>
   </bookViews>
   <sheets>
     <sheet name="JCQ50-ADM022-1-1 - Phieu NKTD" sheetId="1" r:id="rId1"/>
-    <sheet name="Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Data" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'JCQ50-ADM022-1-1 - Phieu NKTD'!$A$1:$P$21</definedName>
@@ -43,10 +43,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="31">
   <si>
     <t xml:space="preserve">PHIẾU NHẬP KHO SẢN PHẨM VÀO KHO TỰ ĐỘNG
 自動倉庫への製品入庫票 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số phiếu/入庫票No： </t>
   </si>
   <si>
     <r>
@@ -434,39 +437,12 @@
   <si>
     <t xml:space="preserve"> /     /</t>
   </si>
-  <si>
-    <t>STT</t>
-  </si>
-  <si>
-    <t>Mã Sản Phẩm</t>
-  </si>
-  <si>
-    <t>Số Lô</t>
-  </si>
-  <si>
-    <t>Mẻ tiệt trùng</t>
-  </si>
-  <si>
-    <t>Thời gian thoát khí</t>
-  </si>
-  <si>
-    <t>Số lượng</t>
-  </si>
-  <si>
-    <t>SoPhieu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Số phiếu/入庫票No： </t>
-  </si>
-  <si>
-    <t>NKTD-TIS-2509-001</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -508,12 +484,6 @@
       <sz val="9"/>
       <name val="MS Mincho"/>
       <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="MS Mincho"/>
-      <family val="3"/>
     </font>
     <font>
       <sz val="9"/>
@@ -535,6 +505,31 @@
       <charset val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <name val="MS Mincho"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="MS Mincho"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="MS Mincho"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -548,35 +543,11 @@
       <family val="1"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <name val="MS Mincho"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="MS Mincho"/>
-      <family val="3"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Wingdings 2"/>
       <family val="1"/>
       <charset val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF0F9ED5"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -766,9 +737,6 @@
   <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -788,31 +756,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
@@ -820,101 +773,121 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -930,121 +903,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>161925</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>255996</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>448797</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{504C9D80-5FF4-49BA-BCF0-0D542ECD90B0}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="161925" y="123825"/>
-          <a:ext cx="1789521" cy="324972"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>123824</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>352425</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>514349</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Rectangle 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C13EBD85-1A45-4845-BAC6-3AE3E34B1BE4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="104775" y="123824"/>
-          <a:ext cx="1943100" cy="390525"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1370,551 +1228,557 @@
   <dimension ref="A1:Q25"/>
   <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.25" style="3" customWidth="1"/>
-    <col min="2" max="2" width="14" style="3" customWidth="1"/>
-    <col min="3" max="3" width="3" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.75" style="3" customWidth="1"/>
-    <col min="5" max="5" width="3" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="3" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="3" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17" style="3" customWidth="1"/>
-    <col min="11" max="12" width="18.625" style="3" customWidth="1"/>
-    <col min="13" max="13" width="16.25" style="3" customWidth="1"/>
-    <col min="14" max="16" width="20.75" style="3" customWidth="1"/>
-    <col min="17" max="17" width="19" style="3" customWidth="1"/>
-    <col min="18" max="16384" width="9.125" style="3"/>
+    <col min="1" max="1" width="5.25" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14" style="2" customWidth="1"/>
+    <col min="3" max="3" width="3" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.75" style="2" customWidth="1"/>
+    <col min="5" max="5" width="3" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="3" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="3" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" style="2" customWidth="1"/>
+    <col min="11" max="12" width="18.625" style="2" customWidth="1"/>
+    <col min="13" max="13" width="16.25" style="2" customWidth="1"/>
+    <col min="14" max="16" width="20.75" style="2" customWidth="1"/>
+    <col min="17" max="17" width="19" style="2" customWidth="1"/>
+    <col min="18" max="23" width="9.125" style="2" customWidth="1"/>
+    <col min="24" max="16384" width="9.125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:17" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
-      <c r="Q1" s="2"/>
-    </row>
-    <row r="2" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="4"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="4"/>
-      <c r="N2" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="O2" s="32" t="str">
+      <c r="Q1" s="1"/>
+    </row>
+    <row r="2" spans="1:17" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="32"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="39"/>
+      <c r="N2" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="O2" s="20" t="str">
         <f>IF(Data!G2&lt;&gt;"",Data!G2,"-")</f>
-        <v>NKTD-TIS-2509-001</v>
-      </c>
-      <c r="Q2" s="7"/>
+        <v>-</v>
+      </c>
+      <c r="Q2" s="6"/>
     </row>
     <row r="3" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="4"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="4"/>
-      <c r="N3" s="6"/>
-      <c r="Q3" s="7"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="3"/>
+      <c r="N3" s="5"/>
+      <c r="Q3" s="6"/>
     </row>
     <row r="4" spans="1:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="9" t="s">
+      <c r="A4" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="9" t="s">
+      <c r="B4" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="9" t="s">
+      <c r="C4" s="51"/>
+      <c r="D4" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="9" t="s">
+      <c r="E4" s="51"/>
+      <c r="F4" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="10"/>
-      <c r="J4" s="8" t="s">
+      <c r="G4" s="51"/>
+      <c r="H4" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="11" t="s">
+      <c r="I4" s="51"/>
+      <c r="J4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="K4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="L4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="11" t="s">
+      <c r="M4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="N4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="P4" s="8" t="s">
+      <c r="O4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="Q4" s="13"/>
+      <c r="P4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q4" s="10"/>
     </row>
     <row r="5" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
+      <c r="A5" s="52" t="str">
         <f>IF(Data!A2&lt;&gt;"",Data!A2,"-")</f>
-        <v>1</v>
-      </c>
-      <c r="B5" s="15">
+        <v>-</v>
+      </c>
+      <c r="B5" s="36" t="str">
         <f>IF(Data!B2&lt;&gt;"",Data!B2,"-")</f>
-        <v>123</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="15">
+        <v>-</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="36" t="str">
         <f>IF(Data!C2&lt;&gt;"",Data!C2,"-")</f>
-        <v>123</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="15">
+        <v>-</v>
+      </c>
+      <c r="E5" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="36" t="str">
         <f>IF(Data!D2&lt;&gt;"",Data!D2,"-")</f>
-        <v>123</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="15">
+        <v>-</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="36" t="str">
         <f>IF(Data!E2&lt;&gt;"",Data!E2,"-")</f>
-        <v>123</v>
-      </c>
-      <c r="I5" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="J5" s="17">
+        <v>-</v>
+      </c>
+      <c r="I5" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="11" t="str">
         <f>IF(Data!F2&lt;&gt;"",Data!F2,"-")</f>
-        <v>123</v>
-      </c>
-      <c r="K5" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="L5" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="M5" s="19"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="P5" s="20"/>
+        <v>-</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="L5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="M5" s="13"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P5" s="14"/>
     </row>
     <row r="6" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21"/>
-      <c r="B6" s="22"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="17" t="str">
+      <c r="A6" s="53"/>
+      <c r="B6" s="37"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="11" t="str">
         <f>IF(Data!F3&lt;&gt;"",Data!F3,"-")</f>
         <v>-</v>
       </c>
-      <c r="K6" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="L6" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="M6" s="19"/>
-      <c r="N6" s="24"/>
-      <c r="O6" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="P6" s="24"/>
+      <c r="K6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="L6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="M6" s="13"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P6" s="16"/>
     </row>
     <row r="7" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="21"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="17" t="str">
+      <c r="A7" s="53"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="11" t="str">
         <f>IF(Data!F4&lt;&gt;"",Data!F4,"-")</f>
         <v>-</v>
       </c>
-      <c r="K7" s="18" t="s">
+      <c r="K7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="L7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="M7" s="13"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P7" s="16"/>
+    </row>
+    <row r="8" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="53"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="L7" s="18" t="s">
+      <c r="D8" s="37"/>
+      <c r="E8" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="M7" s="19"/>
-      <c r="N7" s="24"/>
-      <c r="O7" s="18" t="s">
+      <c r="F8" s="37"/>
+      <c r="G8" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="P7" s="24"/>
-    </row>
-    <row r="8" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-      <c r="B8" s="22"/>
-      <c r="C8" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="22"/>
-      <c r="E8" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" s="22"/>
-      <c r="I8" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="J8" s="17" t="str">
+      <c r="H8" s="37"/>
+      <c r="I8" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="11" t="str">
         <f>IF(Data!F5&lt;&gt;"",Data!F5,"-")</f>
         <v>-</v>
       </c>
-      <c r="K8" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="L8" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="M8" s="19"/>
-      <c r="N8" s="24"/>
-      <c r="O8" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="P8" s="24"/>
+      <c r="K8" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="M8" s="13"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P8" s="16"/>
     </row>
     <row r="9" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="17" t="str">
+      <c r="A9" s="53"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="11" t="str">
         <f>IF(Data!F6&lt;&gt;"",Data!F6,"-")</f>
         <v>-</v>
       </c>
-      <c r="K9" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="L9" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="M9" s="19"/>
-      <c r="N9" s="24"/>
-      <c r="O9" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="P9" s="24"/>
+      <c r="K9" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="L9" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="M9" s="13"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P9" s="16"/>
     </row>
     <row r="10" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="21"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="17" t="str">
+      <c r="A10" s="53"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="11" t="str">
         <f>IF(Data!F7&lt;&gt;"",Data!F7,"-")</f>
         <v>-</v>
       </c>
-      <c r="K10" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="L10" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="M10" s="19"/>
-      <c r="N10" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="O10" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="P10" s="26" t="s">
+      <c r="K10" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="M10" s="13"/>
+      <c r="N10" s="17" t="s">
         <v>16</v>
       </c>
+      <c r="O10" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P10" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="11" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="29"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="17" t="str">
+      <c r="A11" s="54"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="35"/>
+      <c r="J11" s="11" t="str">
         <f>IF(Data!F8&lt;&gt;"",Data!F8,"-")</f>
         <v>-</v>
       </c>
-      <c r="K11" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="L11" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="M11" s="19"/>
-      <c r="N11" s="30"/>
-      <c r="O11" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="P11" s="30"/>
+      <c r="K11" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="L11" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="M11" s="13"/>
+      <c r="N11" s="18"/>
+      <c r="O11" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P11" s="18"/>
     </row>
     <row r="12" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="33"/>
-      <c r="L12" s="33"/>
-      <c r="N12" s="34"/>
-      <c r="O12" s="33"/>
-      <c r="P12" s="34"/>
+      <c r="A12" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="21"/>
+      <c r="L12" s="21"/>
+      <c r="N12" s="22"/>
+      <c r="O12" s="21"/>
+      <c r="P12" s="22"/>
     </row>
     <row r="13" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="35" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="35"/>
-      <c r="L13" s="35"/>
-      <c r="M13" s="35"/>
-      <c r="N13" s="35"/>
-      <c r="O13" s="35"/>
-      <c r="P13" s="35"/>
-      <c r="Q13" s="36"/>
+      <c r="A13" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="46"/>
+      <c r="I13" s="46"/>
+      <c r="J13" s="46"/>
+      <c r="K13" s="46"/>
+      <c r="L13" s="46"/>
+      <c r="M13" s="46"/>
+      <c r="N13" s="46"/>
+      <c r="O13" s="46"/>
+      <c r="P13" s="46"/>
+      <c r="Q13" s="23"/>
     </row>
     <row r="14" spans="1:17" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="37"/>
-      <c r="I14" s="37"/>
-      <c r="J14" s="37"/>
-      <c r="K14" s="37"/>
-      <c r="L14" s="37"/>
-      <c r="M14" s="37"/>
-      <c r="N14" s="37"/>
-      <c r="O14" s="37"/>
-      <c r="P14" s="37"/>
-      <c r="Q14" s="38"/>
+      <c r="A14" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="47"/>
+      <c r="P14" s="47"/>
+      <c r="Q14" s="24"/>
     </row>
     <row r="15" spans="1:17" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="37"/>
-      <c r="J15" s="37"/>
-      <c r="K15" s="37"/>
-      <c r="L15" s="37"/>
-      <c r="M15" s="37"/>
-      <c r="N15" s="37"/>
-      <c r="O15" s="37"/>
-      <c r="P15" s="37"/>
-      <c r="Q15" s="38"/>
+      <c r="A15" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="47"/>
+      <c r="K15" s="47"/>
+      <c r="L15" s="47"/>
+      <c r="M15" s="47"/>
+      <c r="N15" s="47"/>
+      <c r="O15" s="47"/>
+      <c r="P15" s="47"/>
+      <c r="Q15" s="24"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="39"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="39"/>
-      <c r="J16" s="39"/>
-      <c r="K16" s="39"/>
-      <c r="L16" s="39"/>
-      <c r="M16" s="39"/>
-      <c r="N16" s="39"/>
-      <c r="O16" s="39"/>
-      <c r="P16" s="39"/>
-      <c r="Q16" s="40"/>
-    </row>
-    <row r="17" spans="1:17" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="41" t="s">
+      <c r="A16" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="41"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="41"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="41"/>
-      <c r="I17" s="41"/>
-      <c r="J17" s="41"/>
-      <c r="K17" s="41"/>
-      <c r="L17" s="41"/>
-      <c r="M17" s="41"/>
-      <c r="N17" s="41"/>
-      <c r="O17" s="41"/>
-      <c r="P17" s="41"/>
-      <c r="Q17" s="42"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="48"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="48"/>
+      <c r="H16" s="48"/>
+      <c r="I16" s="48"/>
+      <c r="J16" s="48"/>
+      <c r="K16" s="48"/>
+      <c r="L16" s="48"/>
+      <c r="M16" s="48"/>
+      <c r="N16" s="48"/>
+      <c r="O16" s="48"/>
+      <c r="P16" s="48"/>
+      <c r="Q16" s="25"/>
+    </row>
+    <row r="17" spans="1:17" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="49" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="49"/>
+      <c r="L17" s="49"/>
+      <c r="M17" s="49"/>
+      <c r="N17" s="49"/>
+      <c r="O17" s="49"/>
+      <c r="P17" s="49"/>
+      <c r="Q17" s="26"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A18" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="39"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="39"/>
-      <c r="J18" s="39"/>
-      <c r="K18" s="39"/>
-      <c r="L18" s="39"/>
-      <c r="M18" s="39"/>
-      <c r="N18" s="39"/>
-      <c r="O18" s="39"/>
-      <c r="P18" s="39"/>
-      <c r="Q18" s="40"/>
+      <c r="A18" s="48" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="48"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="48"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="48"/>
+      <c r="K18" s="48"/>
+      <c r="L18" s="48"/>
+      <c r="M18" s="48"/>
+      <c r="N18" s="48"/>
+      <c r="O18" s="48"/>
+      <c r="P18" s="48"/>
+      <c r="Q18" s="25"/>
     </row>
     <row r="19" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="44"/>
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:17" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="45" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="46"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
-      <c r="J20" s="47"/>
-      <c r="M20" s="48" t="s">
+      <c r="A20" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="N20" s="48" t="s">
+      <c r="B20" s="41"/>
+      <c r="C20" s="41"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="41"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="42"/>
+      <c r="M20" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="O20" s="12" t="s">
+      <c r="N20" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="P20" s="48" t="s">
+      <c r="O20" s="8" t="s">
         <v>28</v>
       </c>
+      <c r="P20" s="29" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="21" spans="1:17" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="49"/>
-      <c r="B21" s="50"/>
-      <c r="C21" s="50"/>
-      <c r="D21" s="50"/>
-      <c r="E21" s="50"/>
-      <c r="F21" s="50"/>
-      <c r="G21" s="50"/>
-      <c r="H21" s="50"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="51"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="38"/>
-      <c r="M21" s="52" t="s">
-        <v>29</v>
-      </c>
-      <c r="N21" s="52" t="s">
-        <v>29</v>
-      </c>
-      <c r="O21" s="52" t="s">
-        <v>29</v>
-      </c>
-      <c r="P21" s="53" t="s">
-        <v>29</v>
+      <c r="A21" s="43"/>
+      <c r="B21" s="44"/>
+      <c r="C21" s="44"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="44"/>
+      <c r="H21" s="44"/>
+      <c r="I21" s="44"/>
+      <c r="J21" s="45"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="N21" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="O21" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="P21" s="31" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K22" s="34"/>
+      <c r="K22" s="22"/>
     </row>
     <row r="25" spans="1:17" ht="77.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="H1:M2"/>
+    <mergeCell ref="A20:J21"/>
+    <mergeCell ref="A13:P13"/>
     <mergeCell ref="A15:P15"/>
     <mergeCell ref="A16:P16"/>
     <mergeCell ref="A17:P17"/>
     <mergeCell ref="A18:P18"/>
-    <mergeCell ref="A20:J21"/>
-    <mergeCell ref="F5:F11"/>
-    <mergeCell ref="G5:G11"/>
-    <mergeCell ref="H5:H11"/>
-    <mergeCell ref="I5:I11"/>
-    <mergeCell ref="A13:P13"/>
     <mergeCell ref="A14:P14"/>
-    <mergeCell ref="A1:P1"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="F4:G4"/>
@@ -1924,6 +1788,10 @@
     <mergeCell ref="C5:C11"/>
     <mergeCell ref="D5:D11"/>
     <mergeCell ref="E5:E11"/>
+    <mergeCell ref="F5:F11"/>
+    <mergeCell ref="G5:G11"/>
+    <mergeCell ref="H5:H11"/>
+    <mergeCell ref="I5:I11"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3" xr:uid="{757C4A05-F3ED-4ADD-8F4D-CDE3F0C4C0C8}">
@@ -1935,95 +1803,15 @@
   <headerFooter>
     <oddFooter>&amp;L&amp;"Times New Roman,Regular"Mã số quản lý &amp;"MS Mincho,Regular"(書式管理番号)&amp;"Times New Roman,Regular": JCQ50-ADM022-1-Rev6&amp;R&amp;"Times New Roman,Regular"&amp;P/&amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C005029-DCD6-4A51-B653-27CFAE22036F}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="10.25" customWidth="1"/>
-    <col min="2" max="2" width="12.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.75" customWidth="1"/>
-    <col min="7" max="7" width="15.5" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>123</v>
-      </c>
-      <c r="C2">
-        <v>123</v>
-      </c>
-      <c r="D2">
-        <v>123</v>
-      </c>
-      <c r="E2">
-        <v>123</v>
-      </c>
-      <c r="F2">
-        <v>123</v>
-      </c>
-      <c r="G2" s="54" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="G3" s="54"/>
-    </row>
-    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="G4" s="54"/>
-    </row>
-    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="G5" s="54"/>
-    </row>
-    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="G6" s="54"/>
-    </row>
-    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="G7" s="54"/>
-    </row>
-    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="G8" s="54"/>
-    </row>
-    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="G9" s="54"/>
-    </row>
-    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="G10" s="54"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="17" type="noConversion"/>
+  <sheetData/>
+  <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>